<commit_message>
fix generate data bugs
</commit_message>
<xml_diff>
--- a/sqlapp-command/src/test/resources/com/sqlapp/data/db/command/generator/TAB1.xlsx
+++ b/sqlapp-command/src/test/resources/com/sqlapp/data/db/command/generator/TAB1.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\satot\git\sqlapp\sqlapp-command\src\test\resources\com\sqlapp\data\db\command\generator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3185659F-FB4C-4203-95A7-328D430561B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD1DE791-FC02-4C78-ABF4-2AA21A4E35E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5700" yWindow="5736" windowWidth="24612" windowHeight="17532" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5700" yWindow="5736" windowWidth="24612" windowHeight="17532" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Table" sheetId="1" r:id="rId1"/>
@@ -67,7 +67,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="71">
   <si>
     <t>Table Name</t>
   </si>
@@ -219,9 +219,6 @@
     <t>nextAlphaNumeric( 20 )</t>
   </si>
   <si>
-    <t>nextAlphaNumeric( 12 )</t>
-  </si>
-  <si>
     <t>Max Value</t>
   </si>
   <si>
@@ -270,9 +267,6 @@
     <t>_previous.NUMERIC_VALUES_COL + 1</t>
   </si>
   <si>
-    <t>_previous.INTEGER_GROUP_COL + 1</t>
-  </si>
-  <si>
     <t>Values</t>
   </si>
   <si>
@@ -280,6 +274,18 @@
   </si>
   <si>
     <t>'abc'</t>
+    <phoneticPr fontId="23"/>
+  </si>
+  <si>
+    <t>Group1</t>
+    <phoneticPr fontId="23"/>
+  </si>
+  <si>
+    <t>SELECT 123 AS INTEGER_GROUP_COL, 'abc123' AS VARCHAR_GROUP_COL FROM (VALUES(0))
+UNION ALL
+SELECT 456 AS INTEGER_GROUP_COL, 'abc456' AS VARCHAR_GROUP_COL FROM (VALUES(0))
+UNION ALL
+SELECT 789 AS INTEGER_GROUP_COL, 'abc789' AS VARCHAR_GROUP_COL FROM (VALUES(0))</t>
     <phoneticPr fontId="23"/>
   </si>
 </sst>
@@ -461,7 +467,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -533,6 +539,9 @@
     </xf>
     <xf numFmtId="0" fontId="24" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1086,14 +1095,11 @@
       <c r="R3" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="S3" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="T3" s="8" t="s">
-        <v>38</v>
-      </c>
-      <c r="U3" s="8" t="s">
-        <v>38</v>
+      <c r="S3" t="s">
+        <v>69</v>
+      </c>
+      <c r="T3" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:21" ht="23.4" x14ac:dyDescent="0.4">
@@ -1216,14 +1222,10 @@
       <c r="R5" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="S5" s="12" t="s">
-        <v>38</v>
-      </c>
-      <c r="T5" s="12" t="s">
-        <v>38</v>
-      </c>
+      <c r="S5" s="12"/>
+      <c r="T5" s="12"/>
       <c r="U5" s="23" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" spans="1:21" ht="23.4" x14ac:dyDescent="0.4">
@@ -1281,24 +1283,20 @@
       <c r="R6" s="14" t="s">
         <v>49</v>
       </c>
-      <c r="S6" s="14">
-        <v>1</v>
-      </c>
-      <c r="T6" s="14" t="s">
-        <v>50</v>
-      </c>
+      <c r="S6" s="14"/>
+      <c r="T6" s="14"/>
       <c r="U6" s="14"/>
     </row>
     <row r="7" spans="1:21" ht="23.4" x14ac:dyDescent="0.4">
       <c r="A7" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="B7" s="16" t="s">
         <v>51</v>
-      </c>
-      <c r="B7" s="16" t="s">
-        <v>52</v>
       </c>
       <c r="C7" s="16"/>
       <c r="D7" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="E7" s="16">
         <v>127</v>
@@ -1334,48 +1332,46 @@
         <v>1.7976931348623157E+308</v>
       </c>
       <c r="R7" s="16"/>
-      <c r="S7" s="16">
-        <v>2147483647</v>
-      </c>
+      <c r="S7" s="16"/>
       <c r="T7" s="16"/>
       <c r="U7" s="16"/>
     </row>
     <row r="8" spans="1:21" ht="23.4" x14ac:dyDescent="0.4">
       <c r="A8" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="B8" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="B8" s="18" t="s">
+      <c r="C8" s="18" t="s">
         <v>55</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="D8" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="E8" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="E8" s="18" t="s">
+      <c r="F8" s="18" t="s">
         <v>58</v>
       </c>
-      <c r="F8" s="18" t="s">
+      <c r="G8" s="18" t="s">
         <v>59</v>
       </c>
-      <c r="G8" s="18" t="s">
+      <c r="H8" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="H8" s="18" t="s">
+      <c r="I8" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="I8" s="18" t="s">
+      <c r="J8" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="J8" s="18" t="s">
+      <c r="K8" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="L8" s="18" t="s">
         <v>63</v>
-      </c>
-      <c r="K8" s="18" t="s">
-        <v>63</v>
-      </c>
-      <c r="L8" s="18" t="s">
-        <v>64</v>
       </c>
       <c r="M8" s="18" t="s">
         <v>47</v>
@@ -1384,28 +1380,24 @@
         <v>48</v>
       </c>
       <c r="O8" s="18" t="s">
+        <v>64</v>
+      </c>
+      <c r="P8" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="P8" s="18" t="s">
-        <v>66</v>
-      </c>
       <c r="Q8" s="18" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="R8" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="S8" s="18" t="s">
-        <v>67</v>
-      </c>
-      <c r="T8" s="18" t="s">
-        <v>50</v>
-      </c>
+      <c r="S8" s="18"/>
+      <c r="T8" s="18"/>
       <c r="U8" s="18"/>
     </row>
     <row r="9" spans="1:21" ht="23.4" x14ac:dyDescent="0.4">
       <c r="A9" s="19" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B9" s="20"/>
       <c r="C9" s="20"/>
@@ -1437,20 +1429,27 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:A2"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="18" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="22.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="47.69921875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="23.4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:2" ht="23.4" x14ac:dyDescent="0.4">
       <c r="A1" s="21" t="s">
         <v>37</v>
       </c>
+      <c r="B1" t="s">
+        <v>69</v>
+      </c>
     </row>
-    <row r="2" spans="1:1" ht="23.4" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:2" ht="144" x14ac:dyDescent="0.4">
       <c r="A2" s="22" t="s">
-        <v>69</v>
+        <v>67</v>
+      </c>
+      <c r="B2" s="24" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>

</xml_diff>